<commit_message>
Update data.xlsx with new content and revisions
</commit_message>
<xml_diff>
--- a/src/publish/data.xlsx
+++ b/src/publish/data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Bayer\Bayer.LoadData\Bayer.LoadODSData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\New folder\enademoproject\src\publish\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03A4E1B5-2A1E-4ECD-8FD9-A9F18622BBBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27D5D163-E035-41B3-830B-959DE10E0DF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6B258FCD-D826-42E0-B321-CB971A01F84A}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$F$1:$F$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$1:$C$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Sheet2!$B$1:$B$27</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -1898,7 +1898,7 @@
     <col min="21" max="21" width="14.44140625" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="31.77734375" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="18" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="15.77734375" customWidth="1"/>
     <col min="25" max="25" width="26.6640625" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="11.109375" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="15.5546875" bestFit="1" customWidth="1"/>
@@ -1913,6 +1913,8 @@
     <col min="40" max="40" width="47.44140625" bestFit="1" customWidth="1"/>
     <col min="41" max="41" width="35.88671875" bestFit="1" customWidth="1"/>
     <col min="43" max="43" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="13.77734375" bestFit="1" customWidth="1"/>
     <col min="53" max="53" width="45.109375" bestFit="1" customWidth="1"/>
     <col min="56" max="56" width="49.5546875" bestFit="1" customWidth="1"/>
     <col min="59" max="59" width="12.6640625" bestFit="1" customWidth="1"/>
@@ -9914,7 +9916,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="F1:F32" xr:uid="{E1AF9D5F-633B-4593-A18F-1065DF67794C}"/>
+  <autoFilter ref="B1:C32" xr:uid="{E1AF9D5F-633B-4593-A18F-1065DF67794C}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>